<commit_message>
feat(excel): add conditional formatting for open circuit indicator
Add Excel conditional formatting logic to treat infinity symbol (∞) as a valid
open circuit measurement by coloring cells green. This extends the OVERLOAD
handling feature to ensure consistency across all output formats.
</commit_message>
<xml_diff>
--- a/examples/Boreas_2v1 — копия_2026-02-20.xlsx
+++ b/examples/Boreas_2v1 — копия_2026-02-20.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -507,7 +507,7 @@
           <t>1827128.8300000</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>∞</t>
         </is>
@@ -515,6 +515,38 @@
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>2026-02-20 13:06:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>PSN000001111</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>1792.5444200</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>1827075.4800000</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20 13:13:18</t>
         </is>
       </c>
     </row>

</xml_diff>